<commit_message>
added logic to classify lines - not final code.
</commit_message>
<xml_diff>
--- a/non_essential/pocs_prototyping/wall line overlapping with path line use cases.xlsx
+++ b/non_essential/pocs_prototyping/wall line overlapping with path line use cases.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/U34-Bolt/Personal/development/github/trays/non_essential/pocs_prototyping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1D7AE31-4F38-B34C-9CE4-EA605C6DAB93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A03F6854-8BA4-F044-9027-2B4B1F737789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="28200" activeTab="1" xr2:uid="{6B17E38C-5B5E-4043-8C5B-769B1E56F6BE}"/>
   </bookViews>
   <sheets>
     <sheet name="point comparisons" sheetId="3" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="use cases" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet1" sheetId="1" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="53">
   <si>
     <t>for vertical walls</t>
   </si>
@@ -177,20 +177,35 @@
     <t>&gt;</t>
   </si>
   <si>
-    <t>the below image shows each of the use cases above, granted not in the same order… LOL</t>
+    <t>the below image shows each of the use cases above</t>
   </si>
   <si>
     <t>additional info</t>
   </si>
   <si>
     <t>the path line is in black and the wall line is in pink</t>
+  </si>
+  <si>
+    <t>path line</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>y1</t>
+  </si>
+  <si>
+    <t>y2</t>
+  </si>
+  <si>
+    <t>wall line</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -198,8 +213,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="8" tint="0.39997558519241921"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -212,8 +241,38 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -236,20 +295,276 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -262,6 +577,171 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -284,15 +764,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>48846</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>156308</xdr:rowOff>
+      <xdr:colOff>732691</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>87923</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>2487246</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>177899</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>2233245</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>109514</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -315,8 +795,52 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="986692" y="7600462"/>
+          <a:off x="732691" y="10404231"/>
           <a:ext cx="7772400" cy="2278283"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>517770</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>39076</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>2018324</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>92416</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9569D455-A7B5-1DAC-4DCD-77B7B802480D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="517770" y="7483230"/>
+          <a:ext cx="7772400" cy="2720340"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -747,215 +1271,502 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2119E86-F6BB-DC4B-94C0-4B0F858BED7B}">
-  <dimension ref="A1:D23"/>
+  <dimension ref="B1:K23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" customWidth="1"/>
-    <col min="2" max="2" width="35" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35" style="1" customWidth="1"/>
-    <col min="4" max="4" width="49" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" customWidth="1"/>
+    <col min="3" max="3" width="35" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35" style="1" customWidth="1"/>
+    <col min="5" max="5" width="49" customWidth="1"/>
+    <col min="6" max="11" width="5.5" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="2:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+    <row r="2" spans="2:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="F2" s="22" t="s">
+        <v>48</v>
+      </c>
+      <c r="G2" s="23"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="J2" s="18"/>
+      <c r="K2" s="19"/>
+    </row>
+    <row r="3" spans="2:11" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="58" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="58" t="s">
         <v>46</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="59" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A4" s="2">
+      <c r="F3" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="H3" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="I3" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="J3" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="K3" s="21" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" ht="35" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="60">
         <v>1</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="11"/>
+      <c r="E4" s="12" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A5" s="2">
+      <c r="F4" s="25">
+        <v>0</v>
+      </c>
+      <c r="G4" s="55">
+        <v>0</v>
+      </c>
+      <c r="H4" s="56">
+        <v>20</v>
+      </c>
+      <c r="I4" s="25">
+        <v>25</v>
+      </c>
+      <c r="J4" s="55">
+        <v>80</v>
+      </c>
+      <c r="K4" s="56">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" ht="17" x14ac:dyDescent="0.2">
+      <c r="B5" s="61">
         <v>2.1</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="2"/>
-    </row>
-    <row r="6" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A6" s="2">
+      <c r="E5" s="14"/>
+      <c r="F5" s="26">
+        <v>0</v>
+      </c>
+      <c r="G5" s="27">
+        <v>40</v>
+      </c>
+      <c r="H5" s="28">
+        <v>100</v>
+      </c>
+      <c r="I5" s="52">
+        <v>0</v>
+      </c>
+      <c r="J5" s="53">
+        <v>0</v>
+      </c>
+      <c r="K5" s="54">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="62">
         <v>2.2000000000000002</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="2"/>
-    </row>
-    <row r="7" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A7" s="2">
+      <c r="E6" s="16"/>
+      <c r="F6" s="49">
+        <v>0</v>
+      </c>
+      <c r="G6" s="50">
+        <v>0</v>
+      </c>
+      <c r="H6" s="51">
+        <v>20</v>
+      </c>
+      <c r="I6" s="29">
+        <v>0</v>
+      </c>
+      <c r="J6" s="30">
+        <v>40</v>
+      </c>
+      <c r="K6" s="31">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" ht="17" x14ac:dyDescent="0.2">
+      <c r="B7" s="61">
         <v>3.1</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="2"/>
-    </row>
-    <row r="8" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A8" s="2">
+      <c r="E7" s="14"/>
+      <c r="F7" s="26">
+        <v>0</v>
+      </c>
+      <c r="G7" s="27">
+        <v>0</v>
+      </c>
+      <c r="H7" s="28">
+        <v>50</v>
+      </c>
+      <c r="I7" s="52">
+        <v>0</v>
+      </c>
+      <c r="J7" s="53">
+        <v>50</v>
+      </c>
+      <c r="K7" s="54">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="62">
         <v>3.2</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="C8" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="2"/>
-    </row>
-    <row r="9" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A9" s="2">
+      <c r="E8" s="16"/>
+      <c r="F8" s="49">
+        <v>0</v>
+      </c>
+      <c r="G8" s="50">
+        <v>50</v>
+      </c>
+      <c r="H8" s="51">
+        <v>100</v>
+      </c>
+      <c r="I8" s="29">
+        <v>0</v>
+      </c>
+      <c r="J8" s="30">
+        <v>0</v>
+      </c>
+      <c r="K8" s="31">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" ht="34" x14ac:dyDescent="0.2">
+      <c r="B9" s="61">
         <v>4.0999999999999996</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="2"/>
-    </row>
-    <row r="10" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A10" s="2">
+      <c r="E9" s="14"/>
+      <c r="F9" s="26">
+        <v>0</v>
+      </c>
+      <c r="G9" s="27">
+        <v>25</v>
+      </c>
+      <c r="H9" s="28">
+        <v>100</v>
+      </c>
+      <c r="I9" s="52">
+        <v>0</v>
+      </c>
+      <c r="J9" s="53">
+        <v>0</v>
+      </c>
+      <c r="K9" s="54">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" ht="35" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="62">
         <v>4.2</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="2"/>
-    </row>
-    <row r="11" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A11" s="2">
+      <c r="E10" s="16"/>
+      <c r="F10" s="49">
+        <v>0</v>
+      </c>
+      <c r="G10" s="50">
+        <v>0</v>
+      </c>
+      <c r="H10" s="51">
+        <v>75</v>
+      </c>
+      <c r="I10" s="29">
+        <v>0</v>
+      </c>
+      <c r="J10" s="30">
+        <v>25</v>
+      </c>
+      <c r="K10" s="31">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" ht="34" x14ac:dyDescent="0.2">
+      <c r="B11" s="61">
         <v>5.0999999999999996</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="C11" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="D11" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D11" s="2"/>
-    </row>
-    <row r="12" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A12" s="2">
+      <c r="E11" s="14"/>
+      <c r="F11" s="26">
+        <v>0</v>
+      </c>
+      <c r="G11" s="27">
+        <v>0</v>
+      </c>
+      <c r="H11" s="28">
+        <v>50</v>
+      </c>
+      <c r="I11" s="32">
+        <v>0</v>
+      </c>
+      <c r="J11" s="33">
+        <v>0</v>
+      </c>
+      <c r="K11" s="34">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" ht="34" x14ac:dyDescent="0.2">
+      <c r="B12" s="63">
         <v>5.2</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="C12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="D12" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="2"/>
-    </row>
-    <row r="13" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A13" s="2">
+      <c r="E12" s="9"/>
+      <c r="F12" s="41">
+        <v>0</v>
+      </c>
+      <c r="G12" s="42">
+        <v>50</v>
+      </c>
+      <c r="H12" s="43">
+        <v>100</v>
+      </c>
+      <c r="I12" s="35">
+        <v>0</v>
+      </c>
+      <c r="J12" s="36">
+        <v>0</v>
+      </c>
+      <c r="K12" s="37">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" ht="35" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="62">
         <v>5.3</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="C13" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="D13" s="2"/>
-    </row>
-    <row r="14" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A14" s="2">
+      <c r="E13" s="16"/>
+      <c r="F13" s="44">
+        <v>0</v>
+      </c>
+      <c r="G13" s="45">
+        <v>25</v>
+      </c>
+      <c r="H13" s="46">
+        <v>75</v>
+      </c>
+      <c r="I13" s="38">
+        <v>0</v>
+      </c>
+      <c r="J13" s="39">
+        <v>0</v>
+      </c>
+      <c r="K13" s="40">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11" ht="34" x14ac:dyDescent="0.2">
+      <c r="B14" s="61">
         <v>6.1</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="C14" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="D14" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="2"/>
-    </row>
-    <row r="15" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A15" s="2">
+      <c r="E14" s="14"/>
+      <c r="F14" s="32">
+        <v>0</v>
+      </c>
+      <c r="G14" s="33">
+        <v>0</v>
+      </c>
+      <c r="H14" s="34">
+        <v>100</v>
+      </c>
+      <c r="I14" s="26">
+        <v>0</v>
+      </c>
+      <c r="J14" s="27">
+        <v>0</v>
+      </c>
+      <c r="K14" s="28">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="2:11" ht="34" x14ac:dyDescent="0.2">
+      <c r="B15" s="63">
         <v>6.2</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="C15" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="D15" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D15" s="2"/>
-    </row>
-    <row r="16" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A16" s="2">
+      <c r="E15" s="9"/>
+      <c r="F15" s="35">
+        <v>0</v>
+      </c>
+      <c r="G15" s="36">
+        <v>0</v>
+      </c>
+      <c r="H15" s="37">
+        <v>100</v>
+      </c>
+      <c r="I15" s="41">
+        <v>0</v>
+      </c>
+      <c r="J15" s="42">
+        <v>50</v>
+      </c>
+      <c r="K15" s="43">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11" ht="35" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="62">
         <v>6.3</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="C16" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="D16" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="D16" s="2"/>
-    </row>
-    <row r="17" spans="1:4" ht="68" x14ac:dyDescent="0.2">
-      <c r="A17" s="2">
+      <c r="E16" s="16"/>
+      <c r="F16" s="38">
+        <v>0</v>
+      </c>
+      <c r="G16" s="39">
+        <v>0</v>
+      </c>
+      <c r="H16" s="40">
+        <v>100</v>
+      </c>
+      <c r="I16" s="44">
+        <v>0</v>
+      </c>
+      <c r="J16" s="45">
+        <v>25</v>
+      </c>
+      <c r="K16" s="46">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="2:11" ht="69" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="60">
         <v>7</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="C17" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="D17" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="E17" s="12" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B22" s="8" t="s">
+      <c r="F17" s="25">
+        <v>0</v>
+      </c>
+      <c r="G17" s="47">
+        <v>0</v>
+      </c>
+      <c r="H17" s="48">
+        <v>100</v>
+      </c>
+      <c r="I17" s="25">
+        <v>0</v>
+      </c>
+      <c r="J17" s="47">
+        <v>0</v>
+      </c>
+      <c r="K17" s="48">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="C22" s="8" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B23" s="8" t="s">
+    <row r="23" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="C23" s="8" t="s">
         <v>47</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="I2:K2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>